<commit_message>
Product Hub: PORTAL Dot 1 vao roadmap + release v1.10 + bai hoc branch-theo-phan
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/product/Thinksmart-Product-Hub.xlsx
+++ b/product/Thinksmart-Product-Hub.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Không server lưu data khách, không bắt đăng nhập. Nháp = localStorage trình duyệt từng người. Đây là lợi thế privacy + compliance, là nguyên tắc thiết kế chứ không phải tình cờ.</t>
+          <t>Không server lưu data khách. Nháp = localStorage trình duyệt từng người. Từ v1.10 có đăng nhập NỘI BỘ (video học/forum, Supabase) nhưng nguyên tắc không đổi: data KHÁCH không bao giờ lên server. Đây là lợi thế privacy + compliance.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -644,7 +644,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>NOW — làm ngay (mỗi cái vài giờ)</t>
+          <t>PORTAL — trang nội bộ công ty (đang triển khai, mỗi phần 1 branch feat/*)</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr"/>
@@ -657,27 +657,27 @@
       <c r="A3" s="2" t="inlineStr"/>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Nút 'Gửi cho khách' 1 chạm (Web Share API)</t>
+          <t>Khung portal: trang chủ + Tool thành mục con (/tool)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Gửi JPEG/PDF thẳng vào Zalo/Messenger ngay lúc còn ngồi với khách — khoảnh khắc vàng chốt deal</t>
+          <t>Một địa chỉ duy nhất cho cả đội: học – làm – trao đổi; tool cũ giữ nguyên thói quen dùng</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Cần fallback tải file cho desktop</t>
+          <t>Route không dấu / cuối để giữ đường dẫn tương đối của tool</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong v1.10</t>
         </is>
       </c>
     </row>
@@ -685,27 +685,27 @@
       <c r="A4" s="2" t="inlineStr"/>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Chế độ trình bày (ẩn UI, full màn hình)</t>
+          <t>Login email/mật khẩu + phân quyền Admin/Nhân viên (Supabase)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Đưa điện thoại cho khách xem không lộ nút sửa/nháp — chuyên nghiệp</t>
+          <t>Nội dung nội bộ có kiểm soát; nhân viên mới đăng ký → admin duyệt</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Giữ pinch-zoom hoạt động</t>
+          <t>Chờ owner tạo project Supabase + dán key mới BẬT (đang chế độ mở); data khách vẫn không lên server</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong v1.10 (chờ bật)</t>
         </is>
       </c>
     </row>
@@ -713,27 +713,27 @@
       <c r="A5" s="2" t="inlineStr"/>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Sao lưu / khôi phục nháp ra file JSON</t>
+          <t>Thư viện Video học cho sale (YouTube unlisted + Drive)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Chống mất trắng 10 bản nháp khi xoá cache/đổi máy — rủi ro data lớn nhất hiện nay</t>
+          <t>Đào tạo tập trung: admin dán link là cả đội xem được, lọc theo chuyên mục</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nhắc backup định kỳ kín đáo</t>
+          <t>Video Drive phải share 'anyone with link'; RLS chặn người chưa duyệt</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong v1.10</t>
         </is>
       </c>
     </row>
@@ -741,12 +741,12 @@
       <c r="A6" s="2" t="inlineStr"/>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Disclaimer + footer tự động mọi bản xuất</t>
+          <t>Verify đăng nhập end-to-end + push deploy Đợt 1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>'Chỉ mang tính minh hoạ — not a carrier illustration' + tên agent, không tắt được. Lá chắn compliance cho cả đội</t>
+          <t>Đợt 1 lên tool.thinksmartinsurance.com an toàn</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Đối chiếu yêu cầu từng hãng trước khi khoá nội dung</t>
+          <t>Test đủ: đăng ký → duyệt → đăng nhập → video → guard /tool rồi mới push</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -769,22 +769,22 @@
       <c r="A7" s="2" t="inlineStr"/>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>QR code vCard trên name card &amp; proposal</t>
+          <t>Forum nội bộ: đăng tin + bình luận (Đợt 2)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Khách quét là lưu contact; bản chào chuyển tiếp thành name card lan truyền; kèm số license để khách kiểm chứng</t>
+          <t>Thay nhóm chat trôi tin: thông báo mẫu mới, hỏi đáp, kinh nghiệm đọng lại</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Không nhúng data khách vào QR</t>
+          <t>Cần quy ước kiểm duyệt; làm sau khi auth chạy thật</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -797,12 +797,12 @@
       <c r="A8" s="2" t="inlineStr"/>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Thư viện tin nhắn mẫu tiếng Việt (copy 1 chạm)</t>
+          <t>Trang quản lý thành viên cho admin (Đợt 2)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Cảm ơn sau gặp / nhắc hẹn / sinh nhật / xin referral — việc 3 phút còn 10 giây, lời lẽ cả đội nhất quán</t>
+          <t>Duyệt nhân viên 1 chạm ngay trong web, khỏi vào Supabase dashboard</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Cho sửa 1-2 chữ trước khi copy, tránh 'công nghiệp'</t>
+          <t>Làm sau khi có admin thật dùng thử flow duyệt tay</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -824,7 +824,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>NEXT — kế tiếp (vài ngày mỗi cái)</t>
+          <t>NOW — làm ngay (mỗi cái vài giờ)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr"/>
@@ -837,22 +837,22 @@
       <c r="A10" s="2" t="inlineStr"/>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>So sánh 2–3 phương án cạnh nhau</t>
+          <t>Nút 'Gửi cho khách' 1 chạm (Web Share API)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Trả lời 'đóng ít hơn thì sao?' — ghép các nháp thành 1 ảnh so sánh, tâm lý 3 lựa chọn giúp chốt gói giữa</t>
+          <t>Gửi JPEG/PDF thẳng vào Zalo/Messenger ngay lúc còn ngồi với khách — khoảnh khắc vàng chốt deal</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Số liệu PHẢI chép từ illustration hãng + disclaimer; render 8.8MB x3 cần tuần tự</t>
+          <t>Cần fallback tải file cho desktop</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -865,12 +865,12 @@
       <c r="A11" s="2" t="inlineStr"/>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Máy tính nhu cầu bảo vệ DIME</t>
+          <t>Chế độ trình bày (ẩn UI, full màn hình)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Nợ + thu nhập×năm + nhà + học phí con → mệnh giá có căn cứ, bấm là điền vào ô</t>
+          <t>Đưa điện thoại cho khách xem không lộ nút sửa/nháp — chuyên nghiệp</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Ghi rõ 'tham khảo, không phải tư vấn tài chính'</t>
+          <t>Giữ pinch-zoom hoạt động</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -893,12 +893,12 @@
       <c r="A12" s="2" t="inlineStr"/>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Checklist giấy tờ làm hồ sơ theo hãng</t>
+          <t>Sao lưu / khôi phục nháp ra file JSON</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Gửi khách chuẩn bị trước — hẹn ký 1 lần là xong, deal không nguội</t>
+          <t>Chống mất trắng 10 bản nháp khi xoá cache/đổi máy — rủi ro data lớn nhất hiện nay</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Nội dung để file JSON dễ sửa khi hãng đổi yêu cầu</t>
+          <t>Nhắc backup định kỳ kín đáo</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -921,12 +921,12 @@
       <c r="A13" s="2" t="inlineStr"/>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Ghi chú 1 dòng + trạng thái cho từng nháp</t>
+          <t>Disclaimer + footer tự động mọi bản xuất</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Phân vân / Hẹn lại / Đã chốt — bị cắt ngang 2 ngày vẫn nhớ khách đang ở bước nào</t>
+          <t>'Chỉ mang tính minh hoạ — not a carrier illustration' + tên agent, không tắt được. Lá chắn compliance cho cả đội</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Giữ đúng 1 note + 1 trạng thái, KHÔNG phình thành CRM</t>
+          <t>Đối chiếu yêu cầu từng hãng trước khi khoá nội dung</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -949,12 +949,12 @@
       <c r="A14" s="2" t="inlineStr"/>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Bảng tin đội (news.json) + link cài đặt 1 chạm + tour 60s</t>
+          <t>QR code vCard trên name card &amp; proposal</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Cả đội biết mẫu mới/phí mới ngay khi mở tool; onboarding sale mới bằng 1 link Zalo</t>
+          <t>Khách quét là lưu contact; bản chào chuyển tiếp thành name card lan truyền; kèm số license để khách kiểm chứng</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Đưa việc cập nhật news.json vào push-checklist</t>
+          <t>Không nhúng data khách vào QR</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -977,90 +977,90 @@
       <c r="A15" s="2" t="inlineStr"/>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Thẻ giải thích thuật ngữ tiếng Việt (IUL, cash value...)</t>
+          <t>Thư viện tin nhắn mẫu tiếng Việt (copy 1 chạm)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Khúc khó nhất khi tư vấn cộng đồng — mở thẻ hình đẹp chỉ cho khách thay vì nói suông</t>
+          <t>Cảm ơn sau gặp / nhắc hẹn / sinh nhật / xin referral — việc 3 phút còn 10 giây, lời lẽ cả đội nhất quán</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Cho sửa 1-2 chữ trước khi copy, tránh 'công nghiệp'</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>NEXT — kế tiếp (vài ngày mỗi cái)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>So sánh 2–3 phương án cạnh nhau</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Trả lời 'đóng ít hơn thì sao?' — ghép các nháp thành 1 ảnh so sánh, tâm lý 3 lựa chọn giúp chốt gói giữa</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Nội dung trung tính, chủ agency duyệt trước</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Cảnh báo QC mềm trước khi xuất + nhãn Bảo đảm/Không bảo đảm</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Chặn 80% bản chào lỗi (placeholder chưa sửa, thiếu số) + tách rõ số cam kết vs minh hoạ (NAIC #582)</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Chỉ cảnh báo vàng, KHÔNG chặn cứng — sale đang ngồi với khách</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>LATER — nền tảng (đúng tầm nhìn platform)</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr"/>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Số liệu PHẢI chép từ illustration hãng + disclaimer; render 8.8MB x3 cần tuần tự</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr"/>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Mẫu bài đăng Facebook theo hãng</t>
+          <t>Máy tính nhu cầu bảo vệ DIME</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Nguồn khách số 1; tái dùng engine SVG sẵn có; tên+SĐT tự điền từ preset</t>
+          <t>Nợ + thu nhập×năm + nhà + học phí con → mệnh giá có căn cứ, bấm là điền vào ô</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Disclaimer trong mẫu; duyệt bộ đầu bằng skill viet-insurance-ads</t>
+          <t>Ghi rõ 'tham khảo, không phải tư vấn tài chính'</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1073,22 +1073,22 @@
       <c r="A19" s="2" t="inlineStr"/>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Kho video &amp; tài liệu training</t>
+          <t>Checklist giấy tờ làm hồ sơ theo hãng</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Onboarding sale mới ngay trong tool; tái dùng khung Brochure + link YouTube unlisted</t>
+          <t>Gửi khách chuẩn bị trước — hẹn ký 1 lần là xong, deal không nguội</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Không commit MP4 vào repo; nội dung là việc của chủ</t>
+          <t>Nội dung để file JSON dễ sửa khi hãng đổi yêu cầu</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1101,22 +1101,22 @@
       <c r="A20" s="2" t="inlineStr"/>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Field-map theo manifest (hạ tầng)</t>
+          <t>Ghi chú 1 dòng + trạng thái cho từng nháp</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Thêm hãng mới = 15 phút gán nhãn thay vì 1-2 ngày dò toạ độ. LÀM TRƯỚC khi thêm Allianz/mẫu mới</t>
+          <t>Phân vân / Hẹn lại / Đã chốt — bị cắt ngang 2 ngày vẫn nhớ khách đang ở bước nào</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Giữ fallback heuristic cho 4 mẫu cũ, không thì nháp đang dùng vỡ</t>
+          <t>Giữ đúng 1 note + 1 trạng thái, KHÔNG phình thành CRM</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1129,22 +1129,22 @@
       <c r="A21" s="2" t="inlineStr"/>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Mẫu Whole Life / Final Expense</t>
+          <t>Bảng tin đội (news.json) + link cài đặt 1 chạm + tour 60s</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Cộng đồng lớn tuổi hỏi nhiều; layout gần IUL nên tái dùng editor</t>
+          <t>Cả đội biết mẫu mới/phí mới ngay khi mở tool; onboarding sale mới bằng 1 link Zalo</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Làm SAU field-map manifest</t>
+          <t>Đưa việc cập nhật news.json vào push-checklist</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1157,12 +1157,12 @@
       <c r="A22" s="2" t="inlineStr"/>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Xuất song ngữ Việt–Anh</t>
+          <t>Thẻ giải thích thuật ngữ tiếng Việt (IUL, cash value...)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Thuyết phục cả 2 thế hệ trong nhà (con đọc English review giúp bố mẹ)</t>
+          <t>Khúc khó nhất khi tư vấn cộng đồng — mở thẻ hình đẹp chỉ cho khách thay vì nói suông</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Cần thiết kế lại spacing từng mẫu</t>
+          <t>Nội dung trung tính, chủ agency duyệt trước</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1185,12 +1185,12 @@
       <c r="A23" s="2" t="inlineStr"/>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Đếm sử dụng siêu nhẹ (Vercel function → Google Sheet)</t>
+          <t>Cảnh báo QC mềm trước khi xuất + nhãn Bảo đảm/Không bảo đảm</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Biết đội có dùng không, ai 2 tuần im ắng cần kèm. Chỗ DUY NHẤT đáng làm backend nhẹ</t>
+          <t>Chặn 80% bản chào lỗi (placeholder chưa sửa, thiếu số) + tách rõ số cam kết vs minh hoạ (NAIC #582)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>TUYỆT ĐỐI không log data khách; fail-silent</t>
+          <t>Chỉ cảnh báo vàng, KHÔNG chặn cứng — sale đang ngồi với khách</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1212,7 +1212,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>LẰN RANH — không làm</t>
+          <t>LATER — nền tảng (đúng tầm nhìn platform)</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr"/>
@@ -1225,27 +1225,27 @@
       <c r="A25" s="2" t="inlineStr"/>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Tự tính phí / cash value dự phóng</t>
+          <t>Mẫu bài đăng Facebook theo hãng</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Nguồn khách số 1; tái dùng engine SVG sẵn có; tên+SĐT tự điền từ preset</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>KHÔNG BAO GIỜ: illustration IUL phải từ phần mềm hãng phê duyệt (AG 49-A/B). Tool chỉ trình bày số chép sang</t>
+          <t>Disclaimer trong mẫu; duyệt bộ đầu bằng skill viet-insurance-ads</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Nguyên tắc</t>
+          <t>Chưa làm</t>
         </is>
       </c>
     </row>
@@ -1253,27 +1253,27 @@
       <c r="A26" s="2" t="inlineStr"/>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Bảng giá tham khảo tự tra</t>
+          <t>Kho video &amp; tài liệu training</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Onboarding sale mới ngay trong tool; tái dùng khung Brochure + link YouTube unlisted</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Chỉ làm nếu có người CAM KẾT cập nhật số; giá sai mất uy tín + rủi ro compliance</t>
+          <t>Không commit MP4 vào repo; nội dung là việc của chủ</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Hoãn</t>
+          <t>Xong v1.10 — thành trang /videos của Portal</t>
         </is>
       </c>
     </row>
@@ -1281,25 +1281,205 @@
       <c r="A27" s="2" t="inlineStr"/>
       <c r="B27" s="2" t="inlineStr">
         <is>
+          <t>Field-map theo manifest (hạ tầng)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Thêm hãng mới = 15 phút gán nhãn thay vì 1-2 ngày dò toạ độ. LÀM TRƯỚC khi thêm Allianz/mẫu mới</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Giữ fallback heuristic cho 4 mẫu cũ, không thì nháp đang dùng vỡ</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr"/>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Mẫu Whole Life / Final Expense</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Cộng đồng lớn tuổi hỏi nhiều; layout gần IUL nên tái dùng editor</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Làm SAU field-map manifest</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Xuất song ngữ Việt–Anh</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Thuyết phục cả 2 thế hệ trong nhà (con đọc English review giúp bố mẹ)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Cần thiết kế lại spacing từng mẫu</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Đếm sử dụng siêu nhẹ (Vercel function → Google Sheet)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Biết đội có dùng không, ai 2 tuần im ắng cần kèm. Chỗ DUY NHẤT đáng làm backend nhẹ</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>TUYỆT ĐỐI không log data khách; fail-silent</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>LẰN RANH — không làm</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr"/>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Tự tính phí / cash value dự phóng</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>KHÔNG BAO GIỜ: illustration IUL phải từ phần mềm hãng phê duyệt (AG 49-A/B). Tool chỉ trình bày số chép sang</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Nguyên tắc</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Bảng giá tham khảo tự tra</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ làm nếu có người CAM KẾT cập nhật số; giá sai mất uy tín + rủi ro compliance</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Hoãn</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr"/>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
           <t>CRM đầy đủ / server chứa data khách</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Không, trừ khi đánh giá lại có chủ đích khi làm module quản lý khách</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Nguyên tắc</t>
         </is>
@@ -1316,7 +1496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1350,29 +1530,29 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>v1.02</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026</t>
+          <t>19/07/2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Nháp trình duyệt cho site live (draftsMode browser, max 10 bản) · modal dialog đẹp thay alert hệ thống (13+1 chỗ) · tên khách tự điền khi 'Tạo bản cho khách' · fix bug round-trip '$999.99.70'</t>
+          <t>PORTAL Đợt 1 (local, chưa deploy): trang chủ nội bộ mới · Tool chuyển về /tool nguyên vẹn · trang Video học (YouTube/Drive, admin dán link) · Login email/mật khẩu + phân quyền Admin/Nhân viên (Supabase, RLS) · chế độ mở khi chưa dán key · 4 branch feat/* merge lần lượt</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>100 sale dùng đồng thời không cần đăng nhập; data khách an toàn trên máy từng người; đóng PENDING lâu nhất (lưu nháp trên live); bớt 1 bước nhập tay mỗi bản chào.</t>
+          <t>Web từ 'cái tool' thành trang nội bộ công ty: học – làm – trao đổi một chỗ; nền tảng cho Forum Đợt 2; quy trình branch theo phần giúp lỗi phần nào khoanh phần đó.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>v1.01</t>
+          <t>v1.02</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1382,19 +1562,19 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Placeholder chuẩn cho cả 5 mẫu gốc (Nguyen Van An / Texas / (000) 000-0000) · mobile: nút 44px, safe-area iPhone, chặn pull-to-refresh, tap feedback · contrast đạt AA cả 2 theme · pre-push checklist thành quy định</t>
+          <t>Nháp trình duyệt cho site live (draftsMode browser, max 10 bản) · modal dialog đẹp thay alert hệ thống (13+1 chỗ) · tên khách tự điền khi 'Tạo bản cho khách' · fix bug round-trip '$999.99.70'</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Mẫu gốc chuyên nghiệp, hết lộ SĐT thật của team và data test; dùng mượt trên điện thoại — nơi sale làm việc thật; quy trình release có kỷ luật.</t>
+          <t>100 sale dùng đồng thời không cần đăng nhập; data khách an toàn trên máy từng người; đóng PENDING lâu nhất (lưu nháp trên live); bớt 1 bước nhập tay mỗi bản chào.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>v1.00</t>
+          <t>v1.01</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1404,32 +1584,54 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Badge version trong UI · 11 font THẬT (fix 'font bị đổi khi xuất' — bộ woff cũ là đồ giả) · custom domain tool.thinksmartinsurance.com</t>
+          <t>Placeholder chuẩn cho cả 5 mẫu gốc (Nguyen Van An / Texas / (000) 000-0000) · mobile: nút 44px, safe-area iPhone, chặn pull-to-refresh, tap feedback · contrast đạt AA cả 2 theme · pre-push checklist thành quy định</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Bản xuất đúng font trên MỌI máy (kể cả máy sale không cài SF Pro); địa chỉ dễ nhớ để chia sẻ cho đội; phân biệt được bản local vs live.</t>
+          <t>Mẫu gốc chuyên nghiệp, hết lộ SĐT thật của team và data test; dùng mượt trên điện thoại — nơi sale làm việc thật; quy trình release có kỷ luật.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>v1.00</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>17/07/2026</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Badge version trong UI · 11 font THẬT (fix 'font bị đổi khi xuất' — bộ woff cũ là đồ giả) · custom domain tool.thinksmartinsurance.com</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Bản xuất đúng font trên MỌI máy (kể cả máy sale không cài SF Pro); địa chỉ dễ nhớ để chia sẻ cho đội; phân biệt được bản local vs live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>trước v1.00</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>13–16/07/2026</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Rebrand Thinksmart Tool · design system tím + light/dark · 3 công cụ (Proposal / Brochure / Name Card) · workflow 4 bước · master protection + clone cho khách · agent preset tự nhớ · mobile drawer/bottom-sheet · module hoá 5 file JS · audit UI/UX toàn tool</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Từ editor SVG thô thành sản phẩm nội bộ hoàn chỉnh mà sale thật dùng hằng ngày.</t>
         </is>
@@ -1446,7 +1648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1468,24 +1670,24 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>17/07</t>
+          <t>19/07</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Ship xong phải test ROUND-TRIP (lưu → mở lại → so từng field): bug '$999.99 thành $999.99.70' chỉ lộ khi mở lại, nhìn lúc lưu thì mọi thứ đều đẹp.</t>
+          <t>Mỗi phần một branch feat/*, merge --no-ff lần lượt, mỗi trạng thái sau merge phải chạy được (route/redirect tạm nếu phần sau chưa vào) — lỗi phần nào khoanh vùng phần đó.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>17/07</t>
+          <t>19/07</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Snapshot key→value của SVG nhiều tspan phải lưu CẢ DÒNG, và mọi write phải xoá tspan em — nửa vời là data khách sai số tiền.</t>
+          <t>Mở rộng app 1 trang thành nhiều trang: route KHÔNG dấu '/' cuối thì mọi đường dẫn tương đối của trang cũ giữ nguyên; Express non-strict match cả '/tool/' nên phải tự check req.path mà redirect.</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1699,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>100 người dùng đồng thời KHÔNG có nghĩa cần backend. Hỏi 'ai giữ state?': nháp cá nhân thuộc máy sale (localStorage), server chỉ phục vụ mẫu đọc chung.</t>
+          <t>Ship xong phải test ROUND-TRIP (lưu → mở lại → so từng field): bug '$999.99 thành $999.99.70' chỉ lộ khi mở lại, nhìn lúc lưu thì mọi thứ đều đẹp.</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1711,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Dialog tự vẽ phải mở ĐỒNG BỘ (force reflow), đừng qua requestAnimationFrame — tab nền bị throttle là dialog kẹt vô hình.</t>
+          <t>Snapshot key→value của SVG nhiều tspan phải lưu CẢ DÒNG, và mọi write phải xoá tspan em — nửa vời là data khách sai số tiền.</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1723,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>`viewport-fit=cover` mà thiếu env(safe-area-inset-*) là làm nửa việc — nút bấm nằm dưới thanh home iPhone.</t>
+          <t>100 người dùng đồng thời KHÔNG có nghĩa cần backend. Hỏi 'ai giữ state?': nháp cá nhân thuộc máy sale (localStorage), server chỉ phục vụ mẫu đọc chung.</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1735,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Audit touch target phải quét MỌI nút trong vùng, kể cả nút có chữ bị giấu font-size:0 — media query chỉ nâng icon-btn là sót.</t>
+          <t>Dialog tự vẽ phải mở ĐỒNG BỘ (force reflow), đừng qua requestAnimationFrame — tab nền bị throttle là dialog kẹt vô hình.</t>
         </is>
       </c>
     </row>
@@ -1545,41 +1747,65 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Lỗi phát hiện qua accessibility tree phải verify lại bằng textContent thật trước khi sửa — a11y tree có thể hiện attribute title thay vì chữ nhìn thấy.</t>
+          <t>`viewport-fit=cover` mà thiếu env(safe-area-inset-*) là làm nửa việc — nút bấm nằm dưới thanh home iPhone.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>16/07</t>
+          <t>17/07</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>'Chuẩn hoá' một tool đang dùng hằng ngày = siết độ chính xác, KHÔNG đổi look — bản sắc (tím #4F00CA, chấm bi, 4 bước) đã tiêu đúng chỗ.</t>
+          <t>Audit touch target phải quét MỌI nút trong vùng, kể cả nút có chữ bị giấu font-size:0 — media query chỉ nâng icon-btn là sót.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>15/07</t>
+          <t>17/07</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Sale hay bị khách gọi cắt ngang → dirty-state + chấm cam + confirm rời trang + export tự lưu. Thiết kế cho người bị gián đoạn, không phải người ngồi yên.</t>
+          <t>Lỗi phát hiện qua accessibility tree phải verify lại bằng textContent thật trước khi sửa — a11y tree có thể hiện attribute title thay vì chữ nhìn thấy.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>16/07</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>'Chuẩn hoá' một tool đang dùng hằng ngày = siết độ chính xác, KHÔNG đổi look — bản sắc (tím #4F00CA, chấm bi, 4 bước) đã tiêu đúng chỗ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>15/07</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Sale hay bị khách gọi cắt ngang → dirty-state + chấm cam + confirm rời trang + export tự lưu. Thiết kế cho người bị gián đoạn, không phải người ngồi yên.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>15/07</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Người dùng thật ghét nút thừa ('4 nút lằng nhằng') → nút theo ngữ cảnh + tự động hoá preset thay vì thêm lựa chọn.</t>
         </is>

</xml_diff>